<commit_message>
added trait file for the big five
</commit_message>
<xml_diff>
--- a/trait_pairs.xlsx
+++ b/trait_pairs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuqin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tamucs-my.sharepoint.com/personal/yq_c_tamu_edu/Documents/Research/genderBias/GenderBias-SRL-Implementation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A78022E-45C3-4188-A880-B84CA4B14106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{6A78022E-45C3-4188-A880-B84CA4B14106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7688B469-C3CE-4E6E-A712-35246FACD681}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -267,10 +267,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -578,280 +577,279 @@
   <dimension ref="A1:B34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.90625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6328125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="13.90625" customWidth="1"/>
+    <col min="2" max="2" width="16.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
+      <c r="A21" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
+      <c r="A22" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
+      <c r="A23" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
+      <c r="A24" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
+      <c r="A25" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
+      <c r="A26" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
+      <c r="A27" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
+      <c r="A28" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
+      <c r="A29" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
+      <c r="A30" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
+      <c r="A31" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
+      <c r="A32" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
+      <c r="A33" t="s">
         <v>31</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
+      <c r="A34" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" t="s">
         <v>65</v>
       </c>
     </row>

</xml_diff>